<commit_message>
feat: activate GO ICMS via Secretaria da Economia XLSX
CKAN DataStore still lacks ICMS columns; the official monthly Economia workbook publishes ICMS Bruto by municipality for PUBLIC_OPEN ingest with lineage and no tax credit.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/official-snapshots/go-economia-repasses-2024-11.xlsx
+++ b/tests/fixtures/official-snapshots/go-economia-repasses-2024-11.xlsx
@@ -10,40 +10,40 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
-    <t xml:space="preserve">ESTADO DE GOIAS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SECRETARIA DA ECONOMIA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DEMONSTRATIVO  DE  REPASSES AOS  MUNICÍPIOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Período Acumulado: 01/11/2024  a 30/11/2024</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ordem</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MUNICÍPIOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ÍNDICE          ( IPM) (3)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">I P V A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">I P I - E X P O R T A Ç Ã O</t>
-  </si>
-  <si>
-    <t xml:space="preserve">I C M S  </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total geral creditado (sem FUNDEB)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bruto</t>
+    <t>ESTADO DE GOIAS</t>
+  </si>
+  <si>
+    <t>SECRETARIA DA ECONOMIA</t>
+  </si>
+  <si>
+    <t>DEMONSTRATIVO  DE  REPASSES AOS  MUNICÍPIOS</t>
+  </si>
+  <si>
+    <t>Período Acumulado: 01/11/2024  a 30/11/2024</t>
+  </si>
+  <si>
+    <t>Ordem</t>
+  </si>
+  <si>
+    <t>MUNICÍPIOS</t>
+  </si>
+  <si>
+    <t>ÍNDICE          ( IPM) (3)</t>
+  </si>
+  <si>
+    <t>I P V A</t>
+  </si>
+  <si>
+    <t>I P I - E X P O R T A Ç Ã O</t>
+  </si>
+  <si>
+    <t>I C M S  </t>
+  </si>
+  <si>
+    <t>Total geral creditado (sem FUNDEB)</t>
+  </si>
+  <si>
+    <t>Bruto</t>
   </si>
   <si>
     <t xml:space="preserve">FUNDEB 20%
@@ -70,13 +70,13 @@
 Repasse</t>
   </si>
   <si>
-    <t xml:space="preserve">ABADIA DE GOIAS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ABADIANIA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TERRITORIO DESCONHECIDO GO</t>
+    <t>ABADIA DE GOIAS</t>
+  </si>
+  <si>
+    <t>GOIANIA</t>
+  </si>
+  <si>
+    <t>TERRITORIO DESCONHECIDO GO</t>
   </si>
 </sst>
 </file>
@@ -241,40 +241,40 @@
         <v>19</v>
       </c>
       <c r="C9">
-        <v>0.1610951</v>
+        <v>0.5</v>
       </c>
       <c r="D9">
-        <v>156959.44</v>
+        <v>3513965.9</v>
       </c>
       <c r="E9">
-        <v>32041.18</v>
+        <v>700000.0</v>
       </c>
       <c r="F9">
-        <v>124918.26</v>
+        <v>2813965.9</v>
       </c>
       <c r="G9">
-        <v>4982.54</v>
+        <v>1000.0</v>
       </c>
       <c r="H9">
-        <v>996.51</v>
+        <v>200.0</v>
       </c>
       <c r="I9">
-        <v>39.86</v>
+        <v>8.0</v>
       </c>
       <c r="J9">
-        <v>3946.17</v>
+        <v>792.0</v>
       </c>
       <c r="K9">
-        <v>897335.27</v>
+        <v>12500000.0</v>
       </c>
       <c r="L9">
-        <v>179466.99</v>
+        <v>2500000.0</v>
       </c>
       <c r="M9">
-        <v>717868.28</v>
+        <v>10000000.0</v>
       </c>
       <c r="N9">
-        <v>846732.71</v>
+        <v>12815757.9</v>
       </c>
     </row>
     <row r="10">

</xml_diff>